<commit_message>
test: expand the canonical table template for scrolling samples
Extend Players and Items to 30 rows each while preserving the original three
rows and schemas. Include a long final-row name to demonstrate horizontal
overflow. Keep legacy migration-only tests tied to the original fixture data
and cover migration with the expanded template separately.

Document the local sample's fixed bottom horizontal scrollbar, vertical
scrolling and position reset on table selection. Sample UMG assets and editor
authoring helpers remain local and excluded from Git.

Validation: 171 unit tests (168 passed, 3 symlink permission skips), GUI smoke
and compileall passed. Production conversion/import populated both existing
DataTables with 30 rows without rewriting C++ or INI. UE 5.8.3 Editor build,
BP compilation, real PIE cell comparisons, native wheel/scrollbar input to the
last row/column, and stable resets after layout all passed. Packaging/cooking
remain untested.
</commit_message>
<xml_diff>
--- a/Tools/resources/TableTemplate.xlsx
+++ b/Tools/resources/TableTemplate.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Guide" sheetId="1" r:id="R6359eda5a71d4f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="R9d38225fb4344d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="R733710a4568d4846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Guide" sheetId="1" r:id="R2e64ec9ece42428f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="R54c67f23717f4a6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="Rb728133edd0d4362"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -179,6 +179,9 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -814,163 +817,625 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
-      <x:c r="A7" s="30"/>
-      <x:c r="B7" s="30"/>
-      <x:c r="C7" s="30"/>
-      <x:c r="D7" s="2"/>
-      <x:c r="E7" s="2"/>
-      <x:c r="F7" s="2"/>
-      <x:c r="G7" s="2"/>
+      <x:c r="A7" s="30" t="str">
+        <x:v>Player_004</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>샘플 플레이어 004</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>SamplePlayer_004</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="G7" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
-      <x:c r="A8" s="30"/>
-      <x:c r="B8" s="30"/>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="2"/>
-      <x:c r="E8" s="2"/>
-      <x:c r="F8" s="2"/>
-      <x:c r="G8" s="2"/>
+      <x:c r="A8" s="34" t="str">
+        <x:v>Player_005</x:v>
+      </x:c>
+      <x:c r="B8" s="34" t="str">
+        <x:v>샘플 플레이어 005</x:v>
+      </x:c>
+      <x:c r="C8" s="34" t="str">
+        <x:v>SamplePlayer_005</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F8" s="35" t="n">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="G8" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
-      <x:c r="A9" s="30"/>
-      <x:c r="B9" s="30"/>
-      <x:c r="C9" s="30"/>
-      <x:c r="D9" s="2"/>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
-      <x:c r="G9" s="2"/>
+      <x:c r="A9" s="30" t="str">
+        <x:v>Player_006</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>샘플 플레이어 006</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>SamplePlayer_006</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
-      <x:c r="A10" s="30"/>
-      <x:c r="B10" s="30"/>
-      <x:c r="C10" s="30"/>
-      <x:c r="D10" s="2"/>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
-      <x:c r="G10" s="2"/>
+      <x:c r="A10" s="34" t="str">
+        <x:v>Player_007</x:v>
+      </x:c>
+      <x:c r="B10" s="34" t="str">
+        <x:v>샘플 플레이어 007</x:v>
+      </x:c>
+      <x:c r="C10" s="34" t="str">
+        <x:v>SamplePlayer_007</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F10" s="35" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="G10" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
-      <x:c r="A11" s="30"/>
-      <x:c r="B11" s="30"/>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-      <x:c r="G11" s="2"/>
+      <x:c r="A11" s="30" t="str">
+        <x:v>Player_008</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>샘플 플레이어 008</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>SamplePlayer_008</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="n">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
-      <x:c r="A12" s="30"/>
-      <x:c r="B12" s="30"/>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
-      <x:c r="G12" s="2"/>
+      <x:c r="A12" s="34" t="str">
+        <x:v>Player_009</x:v>
+      </x:c>
+      <x:c r="B12" s="34" t="str">
+        <x:v>샘플 플레이어 009</x:v>
+      </x:c>
+      <x:c r="C12" s="34" t="str">
+        <x:v>SamplePlayer_009</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F12" s="35" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G12" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
-      <x:c r="A13" s="31"/>
-      <x:c r="B13" s="31"/>
-      <x:c r="C13" s="31"/>
+      <x:c r="A13" s="30" t="str">
+        <x:v>Player_010</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>샘플 플레이어 010</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>SamplePlayer_010</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="n">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
-      <x:c r="A14" s="31"/>
-      <x:c r="B14" s="31"/>
-      <x:c r="C14" s="31"/>
+      <x:c r="A14" s="34" t="str">
+        <x:v>Player_011</x:v>
+      </x:c>
+      <x:c r="B14" s="34" t="str">
+        <x:v>샘플 플레이어 011</x:v>
+      </x:c>
+      <x:c r="C14" s="34" t="str">
+        <x:v>SamplePlayer_011</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F14" s="35" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="G14" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
-      <x:c r="A15" s="31"/>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
+      <x:c r="A15" s="30" t="str">
+        <x:v>Player_012</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>샘플 플레이어 012</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>SamplePlayer_012</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="n">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
-      <x:c r="A16" s="31"/>
-      <x:c r="B16" s="31"/>
-      <x:c r="C16" s="31"/>
+      <x:c r="A16" s="34" t="str">
+        <x:v>Player_013</x:v>
+      </x:c>
+      <x:c r="B16" s="34" t="str">
+        <x:v>샘플 플레이어 013</x:v>
+      </x:c>
+      <x:c r="C16" s="34" t="str">
+        <x:v>SamplePlayer_013</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F16" s="35" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="G16" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
-      <x:c r="A17" s="31"/>
-      <x:c r="B17" s="31"/>
-      <x:c r="C17" s="31"/>
+      <x:c r="A17" s="30" t="str">
+        <x:v>Player_014</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>샘플 플레이어 014</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>SamplePlayer_014</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
-      <x:c r="A18" s="31"/>
-      <x:c r="B18" s="31"/>
-      <x:c r="C18" s="31"/>
+      <x:c r="A18" s="34" t="str">
+        <x:v>Player_015</x:v>
+      </x:c>
+      <x:c r="B18" s="34" t="str">
+        <x:v>샘플 플레이어 015</x:v>
+      </x:c>
+      <x:c r="C18" s="34" t="str">
+        <x:v>SamplePlayer_015</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F18" s="35" t="n">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="G18" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="31"/>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
+      <x:c r="A19" s="30" t="str">
+        <x:v>Player_016</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>샘플 플레이어 016</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>SamplePlayer_016</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
-      <x:c r="A20" s="31"/>
-      <x:c r="B20" s="31"/>
-      <x:c r="C20" s="31"/>
+      <x:c r="A20" s="34" t="str">
+        <x:v>Player_017</x:v>
+      </x:c>
+      <x:c r="B20" s="34" t="str">
+        <x:v>샘플 플레이어 017</x:v>
+      </x:c>
+      <x:c r="C20" s="34" t="str">
+        <x:v>SamplePlayer_017</x:v>
+      </x:c>
+      <x:c r="D20" s="35" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F20" s="35" t="n">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="G20" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
-      <x:c r="A21" s="31"/>
-      <x:c r="B21" s="31"/>
-      <x:c r="C21" s="31"/>
+      <x:c r="A21" s="30" t="str">
+        <x:v>Player_018</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>샘플 플레이어 018</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>SamplePlayer_018</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
-      <x:c r="A22" s="31"/>
-      <x:c r="B22" s="31"/>
-      <x:c r="C22" s="31"/>
+      <x:c r="A22" s="34" t="str">
+        <x:v>Player_019</x:v>
+      </x:c>
+      <x:c r="B22" s="34" t="str">
+        <x:v>샘플 플레이어 019</x:v>
+      </x:c>
+      <x:c r="C22" s="34" t="str">
+        <x:v>SamplePlayer_019</x:v>
+      </x:c>
+      <x:c r="D22" s="35" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F22" s="35" t="n">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="G22" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
-      <x:c r="A23" s="31"/>
-      <x:c r="B23" s="31"/>
-      <x:c r="C23" s="31"/>
+      <x:c r="A23" s="30" t="str">
+        <x:v>Player_020</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>샘플 플레이어 020</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>SamplePlayer_020</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
-      <x:c r="A24" s="31"/>
-      <x:c r="B24" s="31"/>
-      <x:c r="C24" s="31"/>
+      <x:c r="A24" s="34" t="str">
+        <x:v>Player_021</x:v>
+      </x:c>
+      <x:c r="B24" s="34" t="str">
+        <x:v>샘플 플레이어 021</x:v>
+      </x:c>
+      <x:c r="C24" s="34" t="str">
+        <x:v>SamplePlayer_021</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E24" s="35" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F24" s="35" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="G24" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
-      <x:c r="A25" s="31"/>
-      <x:c r="B25" s="31"/>
-      <x:c r="C25" s="31"/>
+      <x:c r="A25" s="30" t="str">
+        <x:v>Player_022</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>샘플 플레이어 022</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>SamplePlayer_022</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="n">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
-      <x:c r="A26" s="31"/>
-      <x:c r="B26" s="31"/>
-      <x:c r="C26" s="31"/>
+      <x:c r="A26" s="34" t="str">
+        <x:v>Player_023</x:v>
+      </x:c>
+      <x:c r="B26" s="34" t="str">
+        <x:v>샘플 플레이어 023</x:v>
+      </x:c>
+      <x:c r="C26" s="34" t="str">
+        <x:v>SamplePlayer_023</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F26" s="35" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G26" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
-      <x:c r="A27" s="31"/>
-      <x:c r="B27" s="31"/>
-      <x:c r="C27" s="31"/>
+      <x:c r="A27" s="30" t="str">
+        <x:v>Player_024</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>샘플 플레이어 024</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>SamplePlayer_024</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="n">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="G27" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
-      <x:c r="A28" s="31"/>
-      <x:c r="B28" s="31"/>
-      <x:c r="C28" s="31"/>
+      <x:c r="A28" s="34" t="str">
+        <x:v>Player_025</x:v>
+      </x:c>
+      <x:c r="B28" s="34" t="str">
+        <x:v>샘플 플레이어 025</x:v>
+      </x:c>
+      <x:c r="C28" s="34" t="str">
+        <x:v>SamplePlayer_025</x:v>
+      </x:c>
+      <x:c r="D28" s="35" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F28" s="35" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="G28" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
-      <x:c r="A29" s="31"/>
-      <x:c r="B29" s="31"/>
-      <x:c r="C29" s="31"/>
+      <x:c r="A29" s="30" t="str">
+        <x:v>Player_026</x:v>
+      </x:c>
+      <x:c r="B29" s="30" t="str">
+        <x:v>샘플 플레이어 026</x:v>
+      </x:c>
+      <x:c r="C29" s="30" t="str">
+        <x:v>SamplePlayer_026</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="n">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="G29" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
-      <x:c r="A30" s="31"/>
-      <x:c r="B30" s="31"/>
-      <x:c r="C30" s="31"/>
+      <x:c r="A30" s="34" t="str">
+        <x:v>Player_027</x:v>
+      </x:c>
+      <x:c r="B30" s="34" t="str">
+        <x:v>샘플 플레이어 027</x:v>
+      </x:c>
+      <x:c r="C30" s="34" t="str">
+        <x:v>SamplePlayer_027</x:v>
+      </x:c>
+      <x:c r="D30" s="35" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F30" s="35" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="G30" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
-      <x:c r="A31" s="31"/>
-      <x:c r="B31" s="31"/>
-      <x:c r="C31" s="31"/>
+      <x:c r="A31" s="30" t="str">
+        <x:v>Player_028</x:v>
+      </x:c>
+      <x:c r="B31" s="30" t="str">
+        <x:v>샘플 플레이어 028</x:v>
+      </x:c>
+      <x:c r="C31" s="30" t="str">
+        <x:v>SamplePlayer_028</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="G31" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
-      <x:c r="A32" s="31"/>
-      <x:c r="B32" s="31"/>
-      <x:c r="C32" s="31"/>
-    </x:row>
-    <x:row r="33" ht="23" customHeight="1">
-      <x:c r="A33" s="31"/>
-      <x:c r="B33" s="31"/>
-      <x:c r="C33" s="31"/>
+      <x:c r="A32" s="34" t="str">
+        <x:v>Player_029</x:v>
+      </x:c>
+      <x:c r="B32" s="34" t="str">
+        <x:v>샘플 플레이어 029</x:v>
+      </x:c>
+      <x:c r="C32" s="34" t="str">
+        <x:v>SamplePlayer_029</x:v>
+      </x:c>
+      <x:c r="D32" s="35" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E32" s="35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F32" s="35" t="n">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="G32" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="44" customHeight="1">
+      <x:c r="A33" s="30" t="str">
+        <x:v>Player_030</x:v>
+      </x:c>
+      <x:c r="B33" s="40" t="str">
+        <x:v>가로 스크롤 확인용 긴 이름을 가진 샘플 플레이어 030</x:v>
+      </x:c>
+      <x:c r="C33" s="30" t="str">
+        <x:v>SamplePlayer_030</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G33" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="31"/>
@@ -1444,157 +1909,544 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
-      <x:c r="A7" s="30"/>
-      <x:c r="B7" s="30"/>
-      <x:c r="C7" s="30"/>
-      <x:c r="D7" s="2"/>
-      <x:c r="E7" s="2"/>
-      <x:c r="F7" s="2"/>
+      <x:c r="A7" s="30" t="str">
+        <x:v>Item_004</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>샘플 아이템 004</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>SampleItem_004</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
-      <x:c r="A8" s="30"/>
-      <x:c r="B8" s="30"/>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="2"/>
-      <x:c r="E8" s="2"/>
-      <x:c r="F8" s="2"/>
+      <x:c r="A8" s="34" t="str">
+        <x:v>Item_005</x:v>
+      </x:c>
+      <x:c r="B8" s="34" t="str">
+        <x:v>샘플 아이템 005</x:v>
+      </x:c>
+      <x:c r="C8" s="34" t="str">
+        <x:v>SampleItem_005</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="n">
+        <x:v>0.375</x:v>
+      </x:c>
+      <x:c r="F8" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
-      <x:c r="A9" s="30"/>
-      <x:c r="B9" s="30"/>
-      <x:c r="C9" s="30"/>
-      <x:c r="D9" s="2"/>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
+      <x:c r="A9" s="30" t="str">
+        <x:v>Item_006</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>샘플 아이템 006</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>SampleItem_006</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
-      <x:c r="A10" s="30"/>
-      <x:c r="B10" s="30"/>
-      <x:c r="C10" s="30"/>
-      <x:c r="D10" s="2"/>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
+      <x:c r="A10" s="34" t="str">
+        <x:v>Item_007</x:v>
+      </x:c>
+      <x:c r="B10" s="34" t="str">
+        <x:v>샘플 아이템 007</x:v>
+      </x:c>
+      <x:c r="C10" s="34" t="str">
+        <x:v>SampleItem_007</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="n">
+        <x:v>0.625</x:v>
+      </x:c>
+      <x:c r="F10" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
-      <x:c r="A11" s="30"/>
-      <x:c r="B11" s="30"/>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
+      <x:c r="A11" s="30" t="str">
+        <x:v>Item_008</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>샘플 아이템 008</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>SampleItem_008</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
-      <x:c r="A12" s="30"/>
-      <x:c r="B12" s="30"/>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
+      <x:c r="A12" s="34" t="str">
+        <x:v>Item_009</x:v>
+      </x:c>
+      <x:c r="B12" s="34" t="str">
+        <x:v>샘플 아이템 009</x:v>
+      </x:c>
+      <x:c r="C12" s="34" t="str">
+        <x:v>SampleItem_009</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="F12" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
-      <x:c r="A13" s="31"/>
-      <x:c r="B13" s="31"/>
-      <x:c r="C13" s="31"/>
+      <x:c r="A13" s="30" t="str">
+        <x:v>Item_010</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>샘플 아이템 010</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>SampleItem_010</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
-      <x:c r="A14" s="31"/>
-      <x:c r="B14" s="31"/>
-      <x:c r="C14" s="31"/>
+      <x:c r="A14" s="34" t="str">
+        <x:v>Item_011</x:v>
+      </x:c>
+      <x:c r="B14" s="34" t="str">
+        <x:v>샘플 아이템 011</x:v>
+      </x:c>
+      <x:c r="C14" s="34" t="str">
+        <x:v>SampleItem_011</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="n">
+        <x:v>1.125</x:v>
+      </x:c>
+      <x:c r="F14" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
-      <x:c r="A15" s="31"/>
-      <x:c r="B15" s="31"/>
-      <x:c r="C15" s="31"/>
+      <x:c r="A15" s="30" t="str">
+        <x:v>Item_012</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>샘플 아이템 012</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>SampleItem_012</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="n">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
-      <x:c r="A16" s="31"/>
-      <x:c r="B16" s="31"/>
-      <x:c r="C16" s="31"/>
+      <x:c r="A16" s="34" t="str">
+        <x:v>Item_013</x:v>
+      </x:c>
+      <x:c r="B16" s="34" t="str">
+        <x:v>샘플 아이템 013</x:v>
+      </x:c>
+      <x:c r="C16" s="34" t="str">
+        <x:v>SampleItem_013</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="n">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="n">
+        <x:v>1.375</x:v>
+      </x:c>
+      <x:c r="F16" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
-      <x:c r="A17" s="31"/>
-      <x:c r="B17" s="31"/>
-      <x:c r="C17" s="31"/>
+      <x:c r="A17" s="30" t="str">
+        <x:v>Item_014</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>샘플 아이템 014</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>SampleItem_014</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
-      <x:c r="A18" s="31"/>
-      <x:c r="B18" s="31"/>
-      <x:c r="C18" s="31"/>
+      <x:c r="A18" s="34" t="str">
+        <x:v>Item_015</x:v>
+      </x:c>
+      <x:c r="B18" s="34" t="str">
+        <x:v>샘플 아이템 015</x:v>
+      </x:c>
+      <x:c r="C18" s="34" t="str">
+        <x:v>SampleItem_015</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="n">
+        <x:v>1.625</x:v>
+      </x:c>
+      <x:c r="F18" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="31"/>
-      <x:c r="B19" s="31"/>
-      <x:c r="C19" s="31"/>
+      <x:c r="A19" s="30" t="str">
+        <x:v>Item_016</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>샘플 아이템 016</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>SampleItem_016</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
-      <x:c r="A20" s="31"/>
-      <x:c r="B20" s="31"/>
-      <x:c r="C20" s="31"/>
+      <x:c r="A20" s="34" t="str">
+        <x:v>Item_017</x:v>
+      </x:c>
+      <x:c r="B20" s="34" t="str">
+        <x:v>샘플 아이템 017</x:v>
+      </x:c>
+      <x:c r="C20" s="34" t="str">
+        <x:v>SampleItem_017</x:v>
+      </x:c>
+      <x:c r="D20" s="35" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="n">
+        <x:v>1.875</x:v>
+      </x:c>
+      <x:c r="F20" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
-      <x:c r="A21" s="31"/>
-      <x:c r="B21" s="31"/>
-      <x:c r="C21" s="31"/>
+      <x:c r="A21" s="30" t="str">
+        <x:v>Item_018</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>샘플 아이템 018</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>SampleItem_018</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
-      <x:c r="A22" s="31"/>
-      <x:c r="B22" s="31"/>
-      <x:c r="C22" s="31"/>
+      <x:c r="A22" s="34" t="str">
+        <x:v>Item_019</x:v>
+      </x:c>
+      <x:c r="B22" s="34" t="str">
+        <x:v>샘플 아이템 019</x:v>
+      </x:c>
+      <x:c r="C22" s="34" t="str">
+        <x:v>SampleItem_019</x:v>
+      </x:c>
+      <x:c r="D22" s="35" t="n">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="n">
+        <x:v>2.125</x:v>
+      </x:c>
+      <x:c r="F22" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
-      <x:c r="A23" s="31"/>
-      <x:c r="B23" s="31"/>
-      <x:c r="C23" s="31"/>
+      <x:c r="A23" s="30" t="str">
+        <x:v>Item_020</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>샘플 아이템 020</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>SampleItem_020</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="n">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
-      <x:c r="A24" s="31"/>
-      <x:c r="B24" s="31"/>
-      <x:c r="C24" s="31"/>
+      <x:c r="A24" s="34" t="str">
+        <x:v>Item_021</x:v>
+      </x:c>
+      <x:c r="B24" s="34" t="str">
+        <x:v>샘플 아이템 021</x:v>
+      </x:c>
+      <x:c r="C24" s="34" t="str">
+        <x:v>SampleItem_021</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="n">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="E24" s="35" t="n">
+        <x:v>2.375</x:v>
+      </x:c>
+      <x:c r="F24" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
-      <x:c r="A25" s="31"/>
-      <x:c r="B25" s="31"/>
-      <x:c r="C25" s="31"/>
+      <x:c r="A25" s="30" t="str">
+        <x:v>Item_022</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>샘플 아이템 022</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>SampleItem_022</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
-      <x:c r="A26" s="31"/>
-      <x:c r="B26" s="31"/>
-      <x:c r="C26" s="31"/>
+      <x:c r="A26" s="34" t="str">
+        <x:v>Item_023</x:v>
+      </x:c>
+      <x:c r="B26" s="34" t="str">
+        <x:v>샘플 아이템 023</x:v>
+      </x:c>
+      <x:c r="C26" s="34" t="str">
+        <x:v>SampleItem_023</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="n">
+        <x:v>2.625</x:v>
+      </x:c>
+      <x:c r="F26" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
-      <x:c r="A27" s="31"/>
-      <x:c r="B27" s="31"/>
-      <x:c r="C27" s="31"/>
+      <x:c r="A27" s="30" t="str">
+        <x:v>Item_024</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>샘플 아이템 024</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>SampleItem_024</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="n">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="n">
+        <x:v>2.75</x:v>
+      </x:c>
+      <x:c r="F27" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
-      <x:c r="A28" s="31"/>
-      <x:c r="B28" s="31"/>
-      <x:c r="C28" s="31"/>
+      <x:c r="A28" s="34" t="str">
+        <x:v>Item_025</x:v>
+      </x:c>
+      <x:c r="B28" s="34" t="str">
+        <x:v>샘플 아이템 025</x:v>
+      </x:c>
+      <x:c r="C28" s="34" t="str">
+        <x:v>SampleItem_025</x:v>
+      </x:c>
+      <x:c r="D28" s="35" t="n">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="n">
+        <x:v>2.875</x:v>
+      </x:c>
+      <x:c r="F28" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
-      <x:c r="A29" s="31"/>
-      <x:c r="B29" s="31"/>
-      <x:c r="C29" s="31"/>
+      <x:c r="A29" s="30" t="str">
+        <x:v>Item_026</x:v>
+      </x:c>
+      <x:c r="B29" s="30" t="str">
+        <x:v>샘플 아이템 026</x:v>
+      </x:c>
+      <x:c r="C29" s="30" t="str">
+        <x:v>SampleItem_026</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F29" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
-      <x:c r="A30" s="31"/>
-      <x:c r="B30" s="31"/>
-      <x:c r="C30" s="31"/>
+      <x:c r="A30" s="34" t="str">
+        <x:v>Item_027</x:v>
+      </x:c>
+      <x:c r="B30" s="34" t="str">
+        <x:v>샘플 아이템 027</x:v>
+      </x:c>
+      <x:c r="C30" s="34" t="str">
+        <x:v>SampleItem_027</x:v>
+      </x:c>
+      <x:c r="D30" s="35" t="n">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="n">
+        <x:v>3.125</x:v>
+      </x:c>
+      <x:c r="F30" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
-      <x:c r="A31" s="31"/>
-      <x:c r="B31" s="31"/>
-      <x:c r="C31" s="31"/>
+      <x:c r="A31" s="30" t="str">
+        <x:v>Item_028</x:v>
+      </x:c>
+      <x:c r="B31" s="30" t="str">
+        <x:v>샘플 아이템 028</x:v>
+      </x:c>
+      <x:c r="C31" s="30" t="str">
+        <x:v>SampleItem_028</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="n">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="F31" s="22" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
-      <x:c r="A32" s="31"/>
-      <x:c r="B32" s="31"/>
-      <x:c r="C32" s="31"/>
-    </x:row>
-    <x:row r="33" ht="23" customHeight="1">
-      <x:c r="A33" s="31"/>
-      <x:c r="B33" s="31"/>
-      <x:c r="C33" s="31"/>
+      <x:c r="A32" s="34" t="str">
+        <x:v>Item_029</x:v>
+      </x:c>
+      <x:c r="B32" s="34" t="str">
+        <x:v>샘플 아이템 029</x:v>
+      </x:c>
+      <x:c r="C32" s="34" t="str">
+        <x:v>SampleItem_029</x:v>
+      </x:c>
+      <x:c r="D32" s="35" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E32" s="35" t="n">
+        <x:v>3.375</x:v>
+      </x:c>
+      <x:c r="F32" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="44" customHeight="1">
+      <x:c r="A33" s="30" t="str">
+        <x:v>Item_030</x:v>
+      </x:c>
+      <x:c r="B33" s="40" t="str">
+        <x:v>가로 스크롤 확인용 긴 이름을 가진 샘플 아이템 030</x:v>
+      </x:c>
+      <x:c r="C33" s="30" t="str">
+        <x:v>SampleItem_030</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="F33" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="31"/>

</xml_diff>